<commit_message>
feat: add OBE curriculum implementation documentation and tables for SISTEKIN 2026
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_ZCODE/Implementasi_Modul_OBE_SISTEKIN2026_UPDATED.xlsx
+++ b/KURIKULUM2026_ZCODE/Implementasi_Modul_OBE_SISTEKIN2026_UPDATED.xlsx
@@ -4477,7 +4477,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>STI-505 Mobile, STI-701 Platform Eng, FST-714 Skripsi</t>
+          <t>STI-505 Mobile, STI-604 Platform Eng, FST-714 Skripsi</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -4642,7 +4642,7 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>STI-303 UI/UX, STI-505 Mobile, STI-701 Platform Eng, STC-01 UXR</t>
+          <t>STI-303 UI/UX, STI-505 Mobile, STI-604 Platform Eng, STC-01 UXR</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>STI-506 Manpro, STI-702 Startup, STC-06 Digital Product Mgmt</t>
+          <t>STI-506 Manpro, STI-701 Startup, STC-06 Digital Product Mgmt</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -10073,7 +10073,7 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>STI-701</t>
+          <t>STI-604</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
@@ -10083,7 +10083,7 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
@@ -10127,7 +10127,7 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>STI-702</t>
+          <t>STI-701</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
@@ -13607,12 +13607,12 @@
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>FST-610</t>
+          <t>STI-604</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Capstone Project</t>
+          <t>Digital Platform Engineering</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
@@ -13625,63 +13625,31 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="H44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="E44" s="9" t="inlineStr"/>
+      <c r="F44" s="9" t="inlineStr"/>
+      <c r="G44" s="9" t="inlineStr"/>
+      <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="9" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr"/>
       <c r="K44" s="9" t="inlineStr"/>
-      <c r="L44" s="9" t="inlineStr"/>
-      <c r="M44" s="9" t="inlineStr">
+      <c r="L44" s="9" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="N44" s="9" t="inlineStr">
+      <c r="M44" s="9" t="inlineStr"/>
+      <c r="N44" s="9" t="inlineStr"/>
+      <c r="O44" s="9" t="inlineStr"/>
+      <c r="P44" s="9" t="inlineStr"/>
+      <c r="Q44" s="9" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="O44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="P44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="R44" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="R44" s="9" t="inlineStr"/>
       <c r="S44" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -13746,7 +13714,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Digital Platform Engineering</t>
+          <t>Inovasi Teknologi &amp; Startup Digital</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
@@ -13766,36 +13734,32 @@
       <c r="I46" s="9" t="inlineStr"/>
       <c r="J46" s="9" t="inlineStr"/>
       <c r="K46" s="9" t="inlineStr"/>
-      <c r="L46" s="9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="L46" s="9" t="inlineStr"/>
       <c r="M46" s="9" t="inlineStr"/>
       <c r="N46" s="9" t="inlineStr"/>
       <c r="O46" s="9" t="inlineStr"/>
       <c r="P46" s="9" t="inlineStr"/>
-      <c r="Q46" s="9" t="inlineStr">
+      <c r="Q46" s="9" t="inlineStr"/>
+      <c r="R46" s="9" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="R46" s="9" t="inlineStr"/>
       <c r="S46" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>STI-702</t>
+          <t>FST-610</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Inovasi Teknologi &amp; Startup Digital</t>
+          <t>Capstone Project FSTI</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
@@ -13808,19 +13772,55 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr"/>
-      <c r="F47" s="8" t="inlineStr"/>
-      <c r="G47" s="8" t="inlineStr"/>
-      <c r="H47" s="8" t="inlineStr"/>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="I47" s="8" t="inlineStr"/>
       <c r="J47" s="8" t="inlineStr"/>
       <c r="K47" s="8" t="inlineStr"/>
       <c r="L47" s="8" t="inlineStr"/>
-      <c r="M47" s="8" t="inlineStr"/>
-      <c r="N47" s="8" t="inlineStr"/>
-      <c r="O47" s="8" t="inlineStr"/>
-      <c r="P47" s="8" t="inlineStr"/>
-      <c r="Q47" s="8" t="inlineStr"/>
+      <c r="M47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="P47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q47" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="R47" s="8" t="inlineStr">
         <is>
           <t>M</t>
@@ -13828,7 +13828,7 @@
       </c>
       <c r="S47" s="8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -13915,7 +13915,7 @@
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr"/>
@@ -13958,7 +13958,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Skripsi / Capstone TA</t>
+          <t>Skripsi / Tugas Akhir</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
@@ -14065,7 +14065,7 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -14350,7 +14350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15162,12 +15162,12 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>STI-303</t>
+          <t>STI-604</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>UI/UX Design &amp; Prototyping (+P)</t>
+          <t>Digital Platform Engineering (+P)</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -15177,44 +15177,44 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>CPMK3</t>
+          <t>CPMK1</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Mengevaluasi kualitas antarmuka melalui Usability Testing (SUS &amp; Heuristic).</t>
+          <t>Merancang arsitektur microservices dan API gateway untuk platform digital skalabel.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Sub-CPMK3.1</t>
+          <t>Sub-CPMK1.1</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Mengukur skor SUS dan menyusun laporan rekomendasi perbaikan UI/UX berbasis bukti.</t>
+          <t>Mengimplementasikan microservices menggunakan Docker dan API Gateway.</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>KK5</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Laporan evaluasi</t>
+          <t>Lab hands-on</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>STI-701</t>
+          <t>STI-604</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -15229,44 +15229,44 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>CPMK1</t>
+          <t>CPMK2</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Merancang arsitektur microservices dan API gateway untuk platform digital skalabel.</t>
+          <t>Membangun pipeline CI/CD dan Infrastructure as Code untuk deployment otomatis.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Sub-CPMK1.1</t>
+          <t>Sub-CPMK2.1</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Mengimplementasikan microservices menggunakan Docker dan API Gateway.</t>
+          <t>Membangun CI/CD pipeline menggunakan GitHub Actions dan Terraform/Ansible.</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>KK5</t>
         </is>
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>Lab hands-on</t>
+          <t>Project DevOps PjBL</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>40</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>STI-701</t>
+          <t>STI-604</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -15281,22 +15281,22 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>CPMK2</t>
+          <t>CPMK3</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Membangun pipeline CI/CD dan Infrastructure as Code untuk deployment otomatis.</t>
+          <t>Mengevaluasi kinerja dan skalabilitas platform digital dengan load testing.</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Sub-CPMK2.1</t>
+          <t>Sub-CPMK3.1</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Membangun CI/CD pipeline menggunakan GitHub Actions dan Terraform/Ansible.</t>
+          <t>Melakukan load testing menggunakan k6/JMeter dan menganalisis metrik performa.</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -15306,64 +15306,64 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Project DevOps PjBL</t>
+          <t>Project evaluasi</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>STI-701</t>
+          <t>STI-603</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Digital Platform Engineering (+P)</t>
+          <t>Keamanan Informasi Lanjut</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>PL-02</t>
+          <t>PL-05</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>CPMK3</t>
+          <t>CPMK1</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Mengevaluasi kinerja dan skalabilitas platform digital dengan load testing.</t>
+          <t>Menganalisis teknik serangan lanjutan dan mensimulasikan penetration testing dasar.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Sub-CPMK3.1</t>
+          <t>Sub-CPMK1.1</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Melakukan load testing menggunakan k6/JMeter dan menganalisis metrik performa.</t>
+          <t>Mensimulasikan serangan OWASP Top 10 dengan Metasploit/Burp Suite.</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>KK5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Project evaluasi</t>
+          <t>Lab penetration testing</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>25</t>
         </is>
       </c>
     </row>
@@ -15385,37 +15385,37 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>CPMK1</t>
+          <t>CPMK2</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Menganalisis teknik serangan lanjutan dan mensimulasikan penetration testing dasar.</t>
+          <t>Melakukan digital forensics analysis terhadap sistem file dan log jaringan.</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Sub-CPMK1.1</t>
+          <t>Sub-CPMK2.1</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Mensimulasikan serangan OWASP Top 10 dengan Metasploit/Burp Suite.</t>
+          <t>Menganalisis artefak digital dan merekonstruksi kronologi insiden keamanan.</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>KK3</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Lab penetration testing</t>
+          <t>Lab forensik</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>30</t>
         </is>
       </c>
     </row>
@@ -15437,129 +15437,105 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>CPMK2</t>
+          <t>CPMK3</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Melakukan digital forensics analysis terhadap sistem file dan log jaringan.</t>
+          <t>Menyusun kebijakan keamanan informasi organisasi berbasis ISO 27001.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Sub-CPMK2.1</t>
+          <t>Sub-CPMK3.1</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Menganalisis artefak digital dan merekonstruksi kronologi insiden keamanan.</t>
+          <t>Membuat IS Policy Framework dan Risk Register mitigasi berbasis studi kasus.</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
-          <t>KK3</t>
+          <t>KK4</t>
         </is>
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Lab forensik</t>
+          <t>Project kebijakan</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>45</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>STI-603</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Keamanan Informasi Lanjut</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>PL-05</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>CPMK3</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>Menyusun kebijakan keamanan informasi organisasi berbasis ISO 27001.</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Sub-CPMK3.1</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>Membuat IS Policy Framework dan Risk Register mitigasi berbasis studi kasus.</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>KK4</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="inlineStr">
-        <is>
-          <t>Project kebijakan</t>
-        </is>
-      </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Kode MK</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Nama Mata Kuliah</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Total Bobot</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Validasi</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr"/>
+      <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr"/>
+      <c r="H25" s="10" t="inlineStr"/>
+      <c r="I25" s="10" t="inlineStr"/>
+      <c r="J25" s="10" t="inlineStr"/>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Kode MK</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Nama Mata Kuliah</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>Total Bobot</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>Validasi</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr"/>
-      <c r="F26" s="10" t="inlineStr"/>
-      <c r="G26" s="10" t="inlineStr"/>
-      <c r="H26" s="10" t="inlineStr"/>
-      <c r="I26" s="10" t="inlineStr"/>
-      <c r="J26" s="10" t="inlineStr"/>
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>STI-601</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Integrasi Layanan Cerdas Berbasis AI</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr"/>
+      <c r="G26" s="9" t="inlineStr"/>
+      <c r="H26" s="9" t="inlineStr"/>
+      <c r="I26" s="9" t="inlineStr"/>
+      <c r="J26" s="9" t="inlineStr"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>STI-601</t>
+          <t>STI-401</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Integrasi Layanan Cerdas Berbasis AI</t>
+          <t>Machine Learning (+P)</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -15582,12 +15558,12 @@
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>STI-401</t>
+          <t>STI-504</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Machine Learning (+P)</t>
+          <t>Internet of Things (+P)</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -15610,12 +15586,12 @@
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>STI-504</t>
+          <t>STI-303</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Internet of Things (+P)</t>
+          <t>UI/UX Design &amp; Prototyping (+P)</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -15638,12 +15614,12 @@
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>STI-303</t>
+          <t>STI-604</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>UI/UX Design &amp; Prototyping (+P)</t>
+          <t>Digital Platform Engineering (+P)</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -15666,12 +15642,12 @@
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>STI-701</t>
+          <t>STI-603</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Digital Platform Engineering (+P)</t>
+          <t>Keamanan Informasi Lanjut</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -15691,34 +15667,6 @@
       <c r="I31" s="8" t="inlineStr"/>
       <c r="J31" s="8" t="inlineStr"/>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>STI-603</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>Keamanan Informasi Lanjut</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr"/>
-      <c r="F32" s="9" t="inlineStr"/>
-      <c r="G32" s="9" t="inlineStr"/>
-      <c r="H32" s="9" t="inlineStr"/>
-      <c r="I32" s="9" t="inlineStr"/>
-      <c r="J32" s="9" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>